<commit_message>
Starting with Power BI Tools - POWER QUERY
</commit_message>
<xml_diff>
--- a/Power BI/Apocolypse Food Prep.xlsx
+++ b/Power BI/Apocolypse Food Prep.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/579481080490e445/Documents/Power BI Tutorials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omkar\OneDrive\Desktop\Data Analyst\Power BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A4C9D61-390D-4023-BEE6-CEA9014A7CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53FBDD9C-D6CC-41FE-8E51-647183507089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{41A734D2-72BA-4562-B34B-238B193B17BA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{41A734D2-72BA-4562-B34B-238B193B17BA}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Purchase Tracker" sheetId="1" r:id="rId1"/>
+    <sheet name="Pivot Table" sheetId="2" r:id="rId2"/>
+    <sheet name="Purchase Overview" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="23" r:id="rId4"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,7 +32,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -35,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="30">
   <si>
     <t>Store</t>
   </si>
@@ -72,15 +76,69 @@
   <si>
     <t>Canned Vegetables</t>
   </si>
+  <si>
+    <t>Rope</t>
+  </si>
+  <si>
+    <t>Flashlight</t>
+  </si>
+  <si>
+    <t>Duct Tape</t>
+  </si>
+  <si>
+    <t>Water Filter</t>
+  </si>
+  <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Sum of Price</t>
+  </si>
+  <si>
+    <t>Column Labels</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>Apocolypse Food Prep Overview</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Products</t>
+  </si>
+  <si>
+    <t>Costco Total</t>
+  </si>
+  <si>
+    <t>Target Total</t>
+  </si>
+  <si>
+    <t>Walmart Total</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="169" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,13 +154,45 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -117,12 +207,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -138,6 +250,1523 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="OMKAR YELSANGE" refreshedDate="46202.939290277776" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="84" xr:uid="{0626256E-5445-4B75-BD2B-83B526C4BBA2}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:D85" sheet="Purchase Tracker"/>
+  </cacheSource>
+  <cacheFields count="6">
+    <cacheField name="Store" numFmtId="0">
+      <sharedItems count="3">
+        <s v="Walmart"/>
+        <s v="Costco"/>
+        <s v="Target"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Product" numFmtId="0">
+      <sharedItems count="9">
+        <s v="Rice"/>
+        <s v="Dried Beans"/>
+        <s v="Bottled Water "/>
+        <s v="Canned Vegetables"/>
+        <s v="Milk"/>
+        <s v="Rope"/>
+        <s v="Flashlight"/>
+        <s v="Duct Tape"/>
+        <s v="Water Filter"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Price" numFmtId="169">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.65" maxValue="39"/>
+    </cacheField>
+    <cacheField name="Date" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2022-01-01T00:00:00" maxDate="2022-04-02T00:00:00" count="5">
+        <d v="2022-01-01T00:00:00"/>
+        <d v="2022-02-01T00:00:00"/>
+        <d v="2022-03-01T00:00:00"/>
+        <d v="2022-04-01T00:00:00"/>
+        <d v="2022-01-03T00:00:00"/>
+      </sharedItems>
+      <fieldGroup par="5"/>
+    </cacheField>
+    <cacheField name="Days (Date)" numFmtId="0" databaseField="0">
+      <fieldGroup base="3">
+        <rangePr groupBy="days" startDate="2022-01-01T00:00:00" endDate="2022-04-02T00:00:00"/>
+        <groupItems count="368">
+          <s v="&lt;01-01-2022"/>
+          <s v="01-Jan"/>
+          <s v="02-Jan"/>
+          <s v="03-Jan"/>
+          <s v="04-Jan"/>
+          <s v="05-Jan"/>
+          <s v="06-Jan"/>
+          <s v="07-Jan"/>
+          <s v="08-Jan"/>
+          <s v="09-Jan"/>
+          <s v="10-Jan"/>
+          <s v="11-Jan"/>
+          <s v="12-Jan"/>
+          <s v="13-Jan"/>
+          <s v="14-Jan"/>
+          <s v="15-Jan"/>
+          <s v="16-Jan"/>
+          <s v="17-Jan"/>
+          <s v="18-Jan"/>
+          <s v="19-Jan"/>
+          <s v="20-Jan"/>
+          <s v="21-Jan"/>
+          <s v="22-Jan"/>
+          <s v="23-Jan"/>
+          <s v="24-Jan"/>
+          <s v="25-Jan"/>
+          <s v="26-Jan"/>
+          <s v="27-Jan"/>
+          <s v="28-Jan"/>
+          <s v="29-Jan"/>
+          <s v="30-Jan"/>
+          <s v="31-Jan"/>
+          <s v="01-Feb"/>
+          <s v="02-Feb"/>
+          <s v="03-Feb"/>
+          <s v="04-Feb"/>
+          <s v="05-Feb"/>
+          <s v="06-Feb"/>
+          <s v="07-Feb"/>
+          <s v="08-Feb"/>
+          <s v="09-Feb"/>
+          <s v="10-Feb"/>
+          <s v="11-Feb"/>
+          <s v="12-Feb"/>
+          <s v="13-Feb"/>
+          <s v="14-Feb"/>
+          <s v="15-Feb"/>
+          <s v="16-Feb"/>
+          <s v="17-Feb"/>
+          <s v="18-Feb"/>
+          <s v="19-Feb"/>
+          <s v="20-Feb"/>
+          <s v="21-Feb"/>
+          <s v="22-Feb"/>
+          <s v="23-Feb"/>
+          <s v="24-Feb"/>
+          <s v="25-Feb"/>
+          <s v="26-Feb"/>
+          <s v="27-Feb"/>
+          <s v="28-Feb"/>
+          <s v="29-Feb"/>
+          <s v="01-Mar"/>
+          <s v="02-Mar"/>
+          <s v="03-Mar"/>
+          <s v="04-Mar"/>
+          <s v="05-Mar"/>
+          <s v="06-Mar"/>
+          <s v="07-Mar"/>
+          <s v="08-Mar"/>
+          <s v="09-Mar"/>
+          <s v="10-Mar"/>
+          <s v="11-Mar"/>
+          <s v="12-Mar"/>
+          <s v="13-Mar"/>
+          <s v="14-Mar"/>
+          <s v="15-Mar"/>
+          <s v="16-Mar"/>
+          <s v="17-Mar"/>
+          <s v="18-Mar"/>
+          <s v="19-Mar"/>
+          <s v="20-Mar"/>
+          <s v="21-Mar"/>
+          <s v="22-Mar"/>
+          <s v="23-Mar"/>
+          <s v="24-Mar"/>
+          <s v="25-Mar"/>
+          <s v="26-Mar"/>
+          <s v="27-Mar"/>
+          <s v="28-Mar"/>
+          <s v="29-Mar"/>
+          <s v="30-Mar"/>
+          <s v="31-Mar"/>
+          <s v="01-Apr"/>
+          <s v="02-Apr"/>
+          <s v="03-Apr"/>
+          <s v="04-Apr"/>
+          <s v="05-Apr"/>
+          <s v="06-Apr"/>
+          <s v="07-Apr"/>
+          <s v="08-Apr"/>
+          <s v="09-Apr"/>
+          <s v="10-Apr"/>
+          <s v="11-Apr"/>
+          <s v="12-Apr"/>
+          <s v="13-Apr"/>
+          <s v="14-Apr"/>
+          <s v="15-Apr"/>
+          <s v="16-Apr"/>
+          <s v="17-Apr"/>
+          <s v="18-Apr"/>
+          <s v="19-Apr"/>
+          <s v="20-Apr"/>
+          <s v="21-Apr"/>
+          <s v="22-Apr"/>
+          <s v="23-Apr"/>
+          <s v="24-Apr"/>
+          <s v="25-Apr"/>
+          <s v="26-Apr"/>
+          <s v="27-Apr"/>
+          <s v="28-Apr"/>
+          <s v="29-Apr"/>
+          <s v="30-Apr"/>
+          <s v="01-May"/>
+          <s v="02-May"/>
+          <s v="03-May"/>
+          <s v="04-May"/>
+          <s v="05-May"/>
+          <s v="06-May"/>
+          <s v="07-May"/>
+          <s v="08-May"/>
+          <s v="09-May"/>
+          <s v="10-May"/>
+          <s v="11-May"/>
+          <s v="12-May"/>
+          <s v="13-May"/>
+          <s v="14-May"/>
+          <s v="15-May"/>
+          <s v="16-May"/>
+          <s v="17-May"/>
+          <s v="18-May"/>
+          <s v="19-May"/>
+          <s v="20-May"/>
+          <s v="21-May"/>
+          <s v="22-May"/>
+          <s v="23-May"/>
+          <s v="24-May"/>
+          <s v="25-May"/>
+          <s v="26-May"/>
+          <s v="27-May"/>
+          <s v="28-May"/>
+          <s v="29-May"/>
+          <s v="30-May"/>
+          <s v="31-May"/>
+          <s v="01-Jun"/>
+          <s v="02-Jun"/>
+          <s v="03-Jun"/>
+          <s v="04-Jun"/>
+          <s v="05-Jun"/>
+          <s v="06-Jun"/>
+          <s v="07-Jun"/>
+          <s v="08-Jun"/>
+          <s v="09-Jun"/>
+          <s v="10-Jun"/>
+          <s v="11-Jun"/>
+          <s v="12-Jun"/>
+          <s v="13-Jun"/>
+          <s v="14-Jun"/>
+          <s v="15-Jun"/>
+          <s v="16-Jun"/>
+          <s v="17-Jun"/>
+          <s v="18-Jun"/>
+          <s v="19-Jun"/>
+          <s v="20-Jun"/>
+          <s v="21-Jun"/>
+          <s v="22-Jun"/>
+          <s v="23-Jun"/>
+          <s v="24-Jun"/>
+          <s v="25-Jun"/>
+          <s v="26-Jun"/>
+          <s v="27-Jun"/>
+          <s v="28-Jun"/>
+          <s v="29-Jun"/>
+          <s v="30-Jun"/>
+          <s v="01-Jul"/>
+          <s v="02-Jul"/>
+          <s v="03-Jul"/>
+          <s v="04-Jul"/>
+          <s v="05-Jul"/>
+          <s v="06-Jul"/>
+          <s v="07-Jul"/>
+          <s v="08-Jul"/>
+          <s v="09-Jul"/>
+          <s v="10-Jul"/>
+          <s v="11-Jul"/>
+          <s v="12-Jul"/>
+          <s v="13-Jul"/>
+          <s v="14-Jul"/>
+          <s v="15-Jul"/>
+          <s v="16-Jul"/>
+          <s v="17-Jul"/>
+          <s v="18-Jul"/>
+          <s v="19-Jul"/>
+          <s v="20-Jul"/>
+          <s v="21-Jul"/>
+          <s v="22-Jul"/>
+          <s v="23-Jul"/>
+          <s v="24-Jul"/>
+          <s v="25-Jul"/>
+          <s v="26-Jul"/>
+          <s v="27-Jul"/>
+          <s v="28-Jul"/>
+          <s v="29-Jul"/>
+          <s v="30-Jul"/>
+          <s v="31-Jul"/>
+          <s v="01-Aug"/>
+          <s v="02-Aug"/>
+          <s v="03-Aug"/>
+          <s v="04-Aug"/>
+          <s v="05-Aug"/>
+          <s v="06-Aug"/>
+          <s v="07-Aug"/>
+          <s v="08-Aug"/>
+          <s v="09-Aug"/>
+          <s v="10-Aug"/>
+          <s v="11-Aug"/>
+          <s v="12-Aug"/>
+          <s v="13-Aug"/>
+          <s v="14-Aug"/>
+          <s v="15-Aug"/>
+          <s v="16-Aug"/>
+          <s v="17-Aug"/>
+          <s v="18-Aug"/>
+          <s v="19-Aug"/>
+          <s v="20-Aug"/>
+          <s v="21-Aug"/>
+          <s v="22-Aug"/>
+          <s v="23-Aug"/>
+          <s v="24-Aug"/>
+          <s v="25-Aug"/>
+          <s v="26-Aug"/>
+          <s v="27-Aug"/>
+          <s v="28-Aug"/>
+          <s v="29-Aug"/>
+          <s v="30-Aug"/>
+          <s v="31-Aug"/>
+          <s v="01-Sep"/>
+          <s v="02-Sep"/>
+          <s v="03-Sep"/>
+          <s v="04-Sep"/>
+          <s v="05-Sep"/>
+          <s v="06-Sep"/>
+          <s v="07-Sep"/>
+          <s v="08-Sep"/>
+          <s v="09-Sep"/>
+          <s v="10-Sep"/>
+          <s v="11-Sep"/>
+          <s v="12-Sep"/>
+          <s v="13-Sep"/>
+          <s v="14-Sep"/>
+          <s v="15-Sep"/>
+          <s v="16-Sep"/>
+          <s v="17-Sep"/>
+          <s v="18-Sep"/>
+          <s v="19-Sep"/>
+          <s v="20-Sep"/>
+          <s v="21-Sep"/>
+          <s v="22-Sep"/>
+          <s v="23-Sep"/>
+          <s v="24-Sep"/>
+          <s v="25-Sep"/>
+          <s v="26-Sep"/>
+          <s v="27-Sep"/>
+          <s v="28-Sep"/>
+          <s v="29-Sep"/>
+          <s v="30-Sep"/>
+          <s v="01-Oct"/>
+          <s v="02-Oct"/>
+          <s v="03-Oct"/>
+          <s v="04-Oct"/>
+          <s v="05-Oct"/>
+          <s v="06-Oct"/>
+          <s v="07-Oct"/>
+          <s v="08-Oct"/>
+          <s v="09-Oct"/>
+          <s v="10-Oct"/>
+          <s v="11-Oct"/>
+          <s v="12-Oct"/>
+          <s v="13-Oct"/>
+          <s v="14-Oct"/>
+          <s v="15-Oct"/>
+          <s v="16-Oct"/>
+          <s v="17-Oct"/>
+          <s v="18-Oct"/>
+          <s v="19-Oct"/>
+          <s v="20-Oct"/>
+          <s v="21-Oct"/>
+          <s v="22-Oct"/>
+          <s v="23-Oct"/>
+          <s v="24-Oct"/>
+          <s v="25-Oct"/>
+          <s v="26-Oct"/>
+          <s v="27-Oct"/>
+          <s v="28-Oct"/>
+          <s v="29-Oct"/>
+          <s v="30-Oct"/>
+          <s v="31-Oct"/>
+          <s v="01-Nov"/>
+          <s v="02-Nov"/>
+          <s v="03-Nov"/>
+          <s v="04-Nov"/>
+          <s v="05-Nov"/>
+          <s v="06-Nov"/>
+          <s v="07-Nov"/>
+          <s v="08-Nov"/>
+          <s v="09-Nov"/>
+          <s v="10-Nov"/>
+          <s v="11-Nov"/>
+          <s v="12-Nov"/>
+          <s v="13-Nov"/>
+          <s v="14-Nov"/>
+          <s v="15-Nov"/>
+          <s v="16-Nov"/>
+          <s v="17-Nov"/>
+          <s v="18-Nov"/>
+          <s v="19-Nov"/>
+          <s v="20-Nov"/>
+          <s v="21-Nov"/>
+          <s v="22-Nov"/>
+          <s v="23-Nov"/>
+          <s v="24-Nov"/>
+          <s v="25-Nov"/>
+          <s v="26-Nov"/>
+          <s v="27-Nov"/>
+          <s v="28-Nov"/>
+          <s v="29-Nov"/>
+          <s v="30-Nov"/>
+          <s v="01-Dec"/>
+          <s v="02-Dec"/>
+          <s v="03-Dec"/>
+          <s v="04-Dec"/>
+          <s v="05-Dec"/>
+          <s v="06-Dec"/>
+          <s v="07-Dec"/>
+          <s v="08-Dec"/>
+          <s v="09-Dec"/>
+          <s v="10-Dec"/>
+          <s v="11-Dec"/>
+          <s v="12-Dec"/>
+          <s v="13-Dec"/>
+          <s v="14-Dec"/>
+          <s v="15-Dec"/>
+          <s v="16-Dec"/>
+          <s v="17-Dec"/>
+          <s v="18-Dec"/>
+          <s v="19-Dec"/>
+          <s v="20-Dec"/>
+          <s v="21-Dec"/>
+          <s v="22-Dec"/>
+          <s v="23-Dec"/>
+          <s v="24-Dec"/>
+          <s v="25-Dec"/>
+          <s v="26-Dec"/>
+          <s v="27-Dec"/>
+          <s v="28-Dec"/>
+          <s v="29-Dec"/>
+          <s v="30-Dec"/>
+          <s v="31-Dec"/>
+          <s v="&gt;02-04-2022"/>
+        </groupItems>
+      </fieldGroup>
+    </cacheField>
+    <cacheField name="Months (Date)" numFmtId="0" databaseField="0">
+      <fieldGroup base="3">
+        <rangePr groupBy="months" startDate="2022-01-01T00:00:00" endDate="2022-04-02T00:00:00"/>
+        <groupItems count="14">
+          <s v="&lt;01-01-2022"/>
+          <s v="Jan"/>
+          <s v="Feb"/>
+          <s v="Mar"/>
+          <s v="Apr"/>
+          <s v="May"/>
+          <s v="Jun"/>
+          <s v="Jul"/>
+          <s v="Aug"/>
+          <s v="Sep"/>
+          <s v="Oct"/>
+          <s v="Nov"/>
+          <s v="Dec"/>
+          <s v="&gt;02-04-2022"/>
+        </groupItems>
+      </fieldGroup>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="84">
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="25"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="23"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="22.99"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="25.75"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="23.99"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="23.25"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="26.99"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="24.99"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="24.25"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="26.99"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="25.25"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="24.75"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="1"/>
+    <n v="22.99"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="20.99"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="1"/>
+    <n v="23.99"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="1"/>
+    <n v="23.99"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="22.99"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="1"/>
+    <n v="24.99"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="1"/>
+    <n v="24.25"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="22.99"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="1"/>
+    <n v="25.45"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="1"/>
+    <n v="24.49"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="23.99"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="1"/>
+    <n v="25.79"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="2"/>
+    <n v="5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="2"/>
+    <n v="4.25"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <n v="4.99"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="2"/>
+    <n v="5.25"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="2"/>
+    <n v="4.49"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <n v="5.15"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="2"/>
+    <n v="5.45"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="2"/>
+    <n v="4.8"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <n v="5.25"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="2"/>
+    <n v="5.75"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="2"/>
+    <n v="4.8899999999999997"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <n v="5.35"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="3"/>
+    <n v="0.65"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="3"/>
+    <n v="0.85"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="3"/>
+    <n v="0.65"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="3"/>
+    <n v="0.75"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="3"/>
+    <n v="0.85"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="3"/>
+    <n v="0.69"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="3"/>
+    <n v="0.85"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="3"/>
+    <n v="0.85"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="3"/>
+    <n v="0.74"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="3"/>
+    <n v="1"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="3"/>
+    <n v="0.85"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="3"/>
+    <n v="0.79"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="4"/>
+    <n v="2"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="4"/>
+    <n v="2.2999999999999998"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="4"/>
+    <n v="2.2000000000000002"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="4"/>
+    <n v="2.1"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="4"/>
+    <n v="2.4"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="4"/>
+    <n v="2.4500000000000002"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="4"/>
+    <n v="2.4"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="4"/>
+    <n v="2.5"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="4"/>
+    <n v="2.7"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="4"/>
+    <n v="2.9"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="4"/>
+    <n v="2.7"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="4"/>
+    <n v="3"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="5"/>
+    <n v="14"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="5"/>
+    <n v="13.5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="5"/>
+    <n v="15"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="5"/>
+    <n v="14.5"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="5"/>
+    <n v="14"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="5"/>
+    <n v="15.25"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="6"/>
+    <n v="10"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="6"/>
+    <n v="13"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="6"/>
+    <n v="12.5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="6"/>
+    <n v="11"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="6"/>
+    <n v="13"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="6"/>
+    <n v="12.75"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="7"/>
+    <n v="5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="7"/>
+    <n v="5"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="7"/>
+    <n v="6"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="7"/>
+    <n v="5.5"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="7"/>
+    <n v="5.25"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="7"/>
+    <n v="6.25"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="8"/>
+    <n v="39"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="8"/>
+    <n v="29"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="8"/>
+    <n v="38"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="8"/>
+    <n v="39"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="8"/>
+    <n v="31"/>
+    <x v="4"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="8"/>
+    <n v="39"/>
+    <x v="4"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6D8D2089-A7C7-4EF7-80C3-EFC593A2C648}" name="PivotTable2" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:F35" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="6">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="10">
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="7"/>
+        <item x="6"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="169" showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="369">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item sd="0" x="14"/>
+        <item sd="0" x="15"/>
+        <item sd="0" x="16"/>
+        <item sd="0" x="17"/>
+        <item sd="0" x="18"/>
+        <item sd="0" x="19"/>
+        <item sd="0" x="20"/>
+        <item sd="0" x="21"/>
+        <item sd="0" x="22"/>
+        <item sd="0" x="23"/>
+        <item sd="0" x="24"/>
+        <item sd="0" x="25"/>
+        <item sd="0" x="26"/>
+        <item sd="0" x="27"/>
+        <item sd="0" x="28"/>
+        <item sd="0" x="29"/>
+        <item sd="0" x="30"/>
+        <item sd="0" x="31"/>
+        <item sd="0" x="32"/>
+        <item sd="0" x="33"/>
+        <item sd="0" x="34"/>
+        <item sd="0" x="35"/>
+        <item sd="0" x="36"/>
+        <item sd="0" x="37"/>
+        <item sd="0" x="38"/>
+        <item sd="0" x="39"/>
+        <item sd="0" x="40"/>
+        <item sd="0" x="41"/>
+        <item sd="0" x="42"/>
+        <item sd="0" x="43"/>
+        <item sd="0" x="44"/>
+        <item sd="0" x="45"/>
+        <item sd="0" x="46"/>
+        <item sd="0" x="47"/>
+        <item sd="0" x="48"/>
+        <item sd="0" x="49"/>
+        <item sd="0" x="50"/>
+        <item sd="0" x="51"/>
+        <item sd="0" x="52"/>
+        <item sd="0" x="53"/>
+        <item sd="0" x="54"/>
+        <item sd="0" x="55"/>
+        <item sd="0" x="56"/>
+        <item sd="0" x="57"/>
+        <item sd="0" x="58"/>
+        <item sd="0" x="59"/>
+        <item sd="0" x="60"/>
+        <item sd="0" x="61"/>
+        <item sd="0" x="62"/>
+        <item sd="0" x="63"/>
+        <item sd="0" x="64"/>
+        <item sd="0" x="65"/>
+        <item sd="0" x="66"/>
+        <item sd="0" x="67"/>
+        <item sd="0" x="68"/>
+        <item sd="0" x="69"/>
+        <item sd="0" x="70"/>
+        <item sd="0" x="71"/>
+        <item sd="0" x="72"/>
+        <item sd="0" x="73"/>
+        <item sd="0" x="74"/>
+        <item sd="0" x="75"/>
+        <item sd="0" x="76"/>
+        <item sd="0" x="77"/>
+        <item sd="0" x="78"/>
+        <item sd="0" x="79"/>
+        <item sd="0" x="80"/>
+        <item sd="0" x="81"/>
+        <item sd="0" x="82"/>
+        <item sd="0" x="83"/>
+        <item sd="0" x="84"/>
+        <item sd="0" x="85"/>
+        <item sd="0" x="86"/>
+        <item sd="0" x="87"/>
+        <item sd="0" x="88"/>
+        <item sd="0" x="89"/>
+        <item sd="0" x="90"/>
+        <item sd="0" x="91"/>
+        <item sd="0" x="92"/>
+        <item sd="0" x="93"/>
+        <item sd="0" x="94"/>
+        <item sd="0" x="95"/>
+        <item sd="0" x="96"/>
+        <item sd="0" x="97"/>
+        <item sd="0" x="98"/>
+        <item sd="0" x="99"/>
+        <item sd="0" x="100"/>
+        <item sd="0" x="101"/>
+        <item sd="0" x="102"/>
+        <item sd="0" x="103"/>
+        <item sd="0" x="104"/>
+        <item sd="0" x="105"/>
+        <item sd="0" x="106"/>
+        <item sd="0" x="107"/>
+        <item sd="0" x="108"/>
+        <item sd="0" x="109"/>
+        <item sd="0" x="110"/>
+        <item sd="0" x="111"/>
+        <item sd="0" x="112"/>
+        <item sd="0" x="113"/>
+        <item sd="0" x="114"/>
+        <item sd="0" x="115"/>
+        <item sd="0" x="116"/>
+        <item sd="0" x="117"/>
+        <item sd="0" x="118"/>
+        <item sd="0" x="119"/>
+        <item sd="0" x="120"/>
+        <item sd="0" x="121"/>
+        <item sd="0" x="122"/>
+        <item sd="0" x="123"/>
+        <item sd="0" x="124"/>
+        <item sd="0" x="125"/>
+        <item sd="0" x="126"/>
+        <item sd="0" x="127"/>
+        <item sd="0" x="128"/>
+        <item sd="0" x="129"/>
+        <item sd="0" x="130"/>
+        <item sd="0" x="131"/>
+        <item sd="0" x="132"/>
+        <item sd="0" x="133"/>
+        <item sd="0" x="134"/>
+        <item sd="0" x="135"/>
+        <item sd="0" x="136"/>
+        <item sd="0" x="137"/>
+        <item sd="0" x="138"/>
+        <item sd="0" x="139"/>
+        <item sd="0" x="140"/>
+        <item sd="0" x="141"/>
+        <item sd="0" x="142"/>
+        <item sd="0" x="143"/>
+        <item sd="0" x="144"/>
+        <item sd="0" x="145"/>
+        <item sd="0" x="146"/>
+        <item sd="0" x="147"/>
+        <item sd="0" x="148"/>
+        <item sd="0" x="149"/>
+        <item sd="0" x="150"/>
+        <item sd="0" x="151"/>
+        <item sd="0" x="152"/>
+        <item sd="0" x="153"/>
+        <item sd="0" x="154"/>
+        <item sd="0" x="155"/>
+        <item sd="0" x="156"/>
+        <item sd="0" x="157"/>
+        <item sd="0" x="158"/>
+        <item sd="0" x="159"/>
+        <item sd="0" x="160"/>
+        <item sd="0" x="161"/>
+        <item sd="0" x="162"/>
+        <item sd="0" x="163"/>
+        <item sd="0" x="164"/>
+        <item sd="0" x="165"/>
+        <item sd="0" x="166"/>
+        <item sd="0" x="167"/>
+        <item sd="0" x="168"/>
+        <item sd="0" x="169"/>
+        <item sd="0" x="170"/>
+        <item sd="0" x="171"/>
+        <item sd="0" x="172"/>
+        <item sd="0" x="173"/>
+        <item sd="0" x="174"/>
+        <item sd="0" x="175"/>
+        <item sd="0" x="176"/>
+        <item sd="0" x="177"/>
+        <item sd="0" x="178"/>
+        <item sd="0" x="179"/>
+        <item sd="0" x="180"/>
+        <item sd="0" x="181"/>
+        <item sd="0" x="182"/>
+        <item sd="0" x="183"/>
+        <item sd="0" x="184"/>
+        <item sd="0" x="185"/>
+        <item sd="0" x="186"/>
+        <item sd="0" x="187"/>
+        <item sd="0" x="188"/>
+        <item sd="0" x="189"/>
+        <item sd="0" x="190"/>
+        <item sd="0" x="191"/>
+        <item sd="0" x="192"/>
+        <item sd="0" x="193"/>
+        <item sd="0" x="194"/>
+        <item sd="0" x="195"/>
+        <item sd="0" x="196"/>
+        <item sd="0" x="197"/>
+        <item sd="0" x="198"/>
+        <item sd="0" x="199"/>
+        <item sd="0" x="200"/>
+        <item sd="0" x="201"/>
+        <item sd="0" x="202"/>
+        <item sd="0" x="203"/>
+        <item sd="0" x="204"/>
+        <item sd="0" x="205"/>
+        <item sd="0" x="206"/>
+        <item sd="0" x="207"/>
+        <item sd="0" x="208"/>
+        <item sd="0" x="209"/>
+        <item sd="0" x="210"/>
+        <item sd="0" x="211"/>
+        <item sd="0" x="212"/>
+        <item sd="0" x="213"/>
+        <item sd="0" x="214"/>
+        <item sd="0" x="215"/>
+        <item sd="0" x="216"/>
+        <item sd="0" x="217"/>
+        <item sd="0" x="218"/>
+        <item sd="0" x="219"/>
+        <item sd="0" x="220"/>
+        <item sd="0" x="221"/>
+        <item sd="0" x="222"/>
+        <item sd="0" x="223"/>
+        <item sd="0" x="224"/>
+        <item sd="0" x="225"/>
+        <item sd="0" x="226"/>
+        <item sd="0" x="227"/>
+        <item sd="0" x="228"/>
+        <item sd="0" x="229"/>
+        <item sd="0" x="230"/>
+        <item sd="0" x="231"/>
+        <item sd="0" x="232"/>
+        <item sd="0" x="233"/>
+        <item sd="0" x="234"/>
+        <item sd="0" x="235"/>
+        <item sd="0" x="236"/>
+        <item sd="0" x="237"/>
+        <item sd="0" x="238"/>
+        <item sd="0" x="239"/>
+        <item sd="0" x="240"/>
+        <item sd="0" x="241"/>
+        <item sd="0" x="242"/>
+        <item sd="0" x="243"/>
+        <item sd="0" x="244"/>
+        <item sd="0" x="245"/>
+        <item sd="0" x="246"/>
+        <item sd="0" x="247"/>
+        <item sd="0" x="248"/>
+        <item sd="0" x="249"/>
+        <item sd="0" x="250"/>
+        <item sd="0" x="251"/>
+        <item sd="0" x="252"/>
+        <item sd="0" x="253"/>
+        <item sd="0" x="254"/>
+        <item sd="0" x="255"/>
+        <item sd="0" x="256"/>
+        <item sd="0" x="257"/>
+        <item sd="0" x="258"/>
+        <item sd="0" x="259"/>
+        <item sd="0" x="260"/>
+        <item sd="0" x="261"/>
+        <item sd="0" x="262"/>
+        <item sd="0" x="263"/>
+        <item sd="0" x="264"/>
+        <item sd="0" x="265"/>
+        <item sd="0" x="266"/>
+        <item sd="0" x="267"/>
+        <item sd="0" x="268"/>
+        <item sd="0" x="269"/>
+        <item sd="0" x="270"/>
+        <item sd="0" x="271"/>
+        <item sd="0" x="272"/>
+        <item sd="0" x="273"/>
+        <item sd="0" x="274"/>
+        <item sd="0" x="275"/>
+        <item sd="0" x="276"/>
+        <item sd="0" x="277"/>
+        <item sd="0" x="278"/>
+        <item sd="0" x="279"/>
+        <item sd="0" x="280"/>
+        <item sd="0" x="281"/>
+        <item sd="0" x="282"/>
+        <item sd="0" x="283"/>
+        <item sd="0" x="284"/>
+        <item sd="0" x="285"/>
+        <item sd="0" x="286"/>
+        <item sd="0" x="287"/>
+        <item sd="0" x="288"/>
+        <item sd="0" x="289"/>
+        <item sd="0" x="290"/>
+        <item sd="0" x="291"/>
+        <item sd="0" x="292"/>
+        <item sd="0" x="293"/>
+        <item sd="0" x="294"/>
+        <item sd="0" x="295"/>
+        <item sd="0" x="296"/>
+        <item sd="0" x="297"/>
+        <item sd="0" x="298"/>
+        <item sd="0" x="299"/>
+        <item sd="0" x="300"/>
+        <item sd="0" x="301"/>
+        <item sd="0" x="302"/>
+        <item sd="0" x="303"/>
+        <item sd="0" x="304"/>
+        <item sd="0" x="305"/>
+        <item sd="0" x="306"/>
+        <item sd="0" x="307"/>
+        <item sd="0" x="308"/>
+        <item sd="0" x="309"/>
+        <item sd="0" x="310"/>
+        <item sd="0" x="311"/>
+        <item sd="0" x="312"/>
+        <item sd="0" x="313"/>
+        <item sd="0" x="314"/>
+        <item sd="0" x="315"/>
+        <item sd="0" x="316"/>
+        <item sd="0" x="317"/>
+        <item sd="0" x="318"/>
+        <item sd="0" x="319"/>
+        <item sd="0" x="320"/>
+        <item sd="0" x="321"/>
+        <item sd="0" x="322"/>
+        <item sd="0" x="323"/>
+        <item sd="0" x="324"/>
+        <item sd="0" x="325"/>
+        <item sd="0" x="326"/>
+        <item sd="0" x="327"/>
+        <item sd="0" x="328"/>
+        <item sd="0" x="329"/>
+        <item sd="0" x="330"/>
+        <item sd="0" x="331"/>
+        <item sd="0" x="332"/>
+        <item sd="0" x="333"/>
+        <item sd="0" x="334"/>
+        <item sd="0" x="335"/>
+        <item sd="0" x="336"/>
+        <item sd="0" x="337"/>
+        <item sd="0" x="338"/>
+        <item sd="0" x="339"/>
+        <item sd="0" x="340"/>
+        <item sd="0" x="341"/>
+        <item sd="0" x="342"/>
+        <item sd="0" x="343"/>
+        <item sd="0" x="344"/>
+        <item sd="0" x="345"/>
+        <item sd="0" x="346"/>
+        <item sd="0" x="347"/>
+        <item sd="0" x="348"/>
+        <item sd="0" x="349"/>
+        <item sd="0" x="350"/>
+        <item sd="0" x="351"/>
+        <item sd="0" x="352"/>
+        <item sd="0" x="353"/>
+        <item sd="0" x="354"/>
+        <item sd="0" x="355"/>
+        <item sd="0" x="356"/>
+        <item sd="0" x="357"/>
+        <item sd="0" x="358"/>
+        <item sd="0" x="359"/>
+        <item sd="0" x="360"/>
+        <item sd="0" x="361"/>
+        <item sd="0" x="362"/>
+        <item sd="0" x="363"/>
+        <item sd="0" x="364"/>
+        <item sd="0" x="365"/>
+        <item sd="0" x="366"/>
+        <item sd="0" x="367"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="15">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="0"/>
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="31">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="5"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Price" fld="2" baseField="0" baseItem="0" numFmtId="169"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -437,20 +2066,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C502D15-4E0D-42D8-A877-22E48FDC669F}">
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D85"/>
   <sheetFormatPr defaultColWidth="15.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="15.88671875" style="2"/>
+    <col min="3" max="3" width="15.88671875" style="8"/>
+    <col min="4" max="4" width="15.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
@@ -464,7 +2094,7 @@
       <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="8">
         <v>25</v>
       </c>
       <c r="D2" s="1">
@@ -478,7 +2108,7 @@
       <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="8">
         <v>23</v>
       </c>
       <c r="D3" s="1">
@@ -492,7 +2122,7 @@
       <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="8">
         <v>22.99</v>
       </c>
       <c r="D4" s="1">
@@ -506,7 +2136,7 @@
       <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="8">
         <v>25.75</v>
       </c>
       <c r="D5" s="1">
@@ -520,7 +2150,7 @@
       <c r="B6" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="8">
         <v>23.99</v>
       </c>
       <c r="D6" s="1">
@@ -534,7 +2164,7 @@
       <c r="B7" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="8">
         <v>23.25</v>
       </c>
       <c r="D7" s="1">
@@ -548,7 +2178,7 @@
       <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="8">
         <v>26.99</v>
       </c>
       <c r="D8" s="1">
@@ -562,7 +2192,7 @@
       <c r="B9" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="8">
         <v>24.99</v>
       </c>
       <c r="D9" s="1">
@@ -576,7 +2206,7 @@
       <c r="B10" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="8">
         <v>24.25</v>
       </c>
       <c r="D10" s="1">
@@ -590,7 +2220,7 @@
       <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="8">
         <v>26.99</v>
       </c>
       <c r="D11" s="1">
@@ -604,7 +2234,7 @@
       <c r="B12" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="8">
         <v>25.25</v>
       </c>
       <c r="D12" s="1">
@@ -618,7 +2248,7 @@
       <c r="B13" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="8">
         <v>24.75</v>
       </c>
       <c r="D13" s="1">
@@ -632,7 +2262,7 @@
       <c r="B14" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="8">
         <v>22.99</v>
       </c>
       <c r="D14" s="1">
@@ -646,7 +2276,7 @@
       <c r="B15" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="8">
         <v>20.99</v>
       </c>
       <c r="D15" s="1">
@@ -660,7 +2290,7 @@
       <c r="B16" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="8">
         <v>23.99</v>
       </c>
       <c r="D16" s="1">
@@ -674,7 +2304,7 @@
       <c r="B17" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="8">
         <v>23.99</v>
       </c>
       <c r="D17" s="1">
@@ -688,7 +2318,7 @@
       <c r="B18" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="8">
         <v>22.99</v>
       </c>
       <c r="D18" s="1">
@@ -702,7 +2332,7 @@
       <c r="B19" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="8">
         <v>24.99</v>
       </c>
       <c r="D19" s="1">
@@ -716,7 +2346,7 @@
       <c r="B20" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="8">
         <v>24.25</v>
       </c>
       <c r="D20" s="1">
@@ -730,7 +2360,7 @@
       <c r="B21" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="8">
         <v>22.99</v>
       </c>
       <c r="D21" s="1">
@@ -744,7 +2374,7 @@
       <c r="B22" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="8">
         <v>25.45</v>
       </c>
       <c r="D22" s="1">
@@ -758,7 +2388,7 @@
       <c r="B23" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="8">
         <v>24.49</v>
       </c>
       <c r="D23" s="1">
@@ -772,7 +2402,7 @@
       <c r="B24" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="8">
         <v>23.99</v>
       </c>
       <c r="D24" s="1">
@@ -786,7 +2416,7 @@
       <c r="B25" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C25" s="8">
         <v>25.79</v>
       </c>
       <c r="D25" s="1">
@@ -800,7 +2430,7 @@
       <c r="B26" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C26" s="8">
         <v>5</v>
       </c>
       <c r="D26" s="1">
@@ -814,7 +2444,7 @@
       <c r="B27" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="2">
+      <c r="C27" s="8">
         <v>4.25</v>
       </c>
       <c r="D27" s="1">
@@ -828,7 +2458,7 @@
       <c r="B28" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="2">
+      <c r="C28" s="8">
         <v>4.99</v>
       </c>
       <c r="D28" s="1">
@@ -842,7 +2472,7 @@
       <c r="B29" t="s">
         <v>7</v>
       </c>
-      <c r="C29" s="2">
+      <c r="C29" s="8">
         <v>5.25</v>
       </c>
       <c r="D29" s="1">
@@ -856,7 +2486,7 @@
       <c r="B30" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="2">
+      <c r="C30" s="8">
         <v>4.49</v>
       </c>
       <c r="D30" s="1">
@@ -870,7 +2500,7 @@
       <c r="B31" t="s">
         <v>7</v>
       </c>
-      <c r="C31" s="2">
+      <c r="C31" s="8">
         <v>5.15</v>
       </c>
       <c r="D31" s="1">
@@ -884,7 +2514,7 @@
       <c r="B32" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="2">
+      <c r="C32" s="8">
         <v>5.45</v>
       </c>
       <c r="D32" s="1">
@@ -898,7 +2528,7 @@
       <c r="B33" t="s">
         <v>7</v>
       </c>
-      <c r="C33" s="2">
+      <c r="C33" s="8">
         <v>4.8</v>
       </c>
       <c r="D33" s="1">
@@ -912,7 +2542,7 @@
       <c r="B34" t="s">
         <v>7</v>
       </c>
-      <c r="C34" s="2">
+      <c r="C34" s="8">
         <v>5.25</v>
       </c>
       <c r="D34" s="1">
@@ -926,7 +2556,7 @@
       <c r="B35" t="s">
         <v>7</v>
       </c>
-      <c r="C35" s="2">
+      <c r="C35" s="8">
         <v>5.75</v>
       </c>
       <c r="D35" s="1">
@@ -940,7 +2570,7 @@
       <c r="B36" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="2">
+      <c r="C36" s="8">
         <v>4.8899999999999997</v>
       </c>
       <c r="D36" s="1">
@@ -954,7 +2584,7 @@
       <c r="B37" t="s">
         <v>7</v>
       </c>
-      <c r="C37" s="2">
+      <c r="C37" s="8">
         <v>5.35</v>
       </c>
       <c r="D37" s="1">
@@ -968,7 +2598,7 @@
       <c r="B38" t="s">
         <v>11</v>
       </c>
-      <c r="C38" s="2">
+      <c r="C38" s="8">
         <v>0.65</v>
       </c>
       <c r="D38" s="1">
@@ -982,7 +2612,7 @@
       <c r="B39" t="s">
         <v>11</v>
       </c>
-      <c r="C39" s="2">
+      <c r="C39" s="8">
         <v>0.85</v>
       </c>
       <c r="D39" s="1">
@@ -996,7 +2626,7 @@
       <c r="B40" t="s">
         <v>11</v>
       </c>
-      <c r="C40" s="2">
+      <c r="C40" s="8">
         <v>0.65</v>
       </c>
       <c r="D40" s="1">
@@ -1010,7 +2640,7 @@
       <c r="B41" t="s">
         <v>11</v>
       </c>
-      <c r="C41" s="2">
+      <c r="C41" s="8">
         <v>0.75</v>
       </c>
       <c r="D41" s="1">
@@ -1024,7 +2654,7 @@
       <c r="B42" t="s">
         <v>11</v>
       </c>
-      <c r="C42" s="2">
+      <c r="C42" s="8">
         <v>0.85</v>
       </c>
       <c r="D42" s="1">
@@ -1038,7 +2668,7 @@
       <c r="B43" t="s">
         <v>11</v>
       </c>
-      <c r="C43" s="2">
+      <c r="C43" s="8">
         <v>0.69</v>
       </c>
       <c r="D43" s="1">
@@ -1052,7 +2682,7 @@
       <c r="B44" t="s">
         <v>11</v>
       </c>
-      <c r="C44" s="2">
+      <c r="C44" s="8">
         <v>0.85</v>
       </c>
       <c r="D44" s="1">
@@ -1066,7 +2696,7 @@
       <c r="B45" t="s">
         <v>11</v>
       </c>
-      <c r="C45" s="2">
+      <c r="C45" s="8">
         <v>0.85</v>
       </c>
       <c r="D45" s="1">
@@ -1080,7 +2710,7 @@
       <c r="B46" t="s">
         <v>11</v>
       </c>
-      <c r="C46" s="2">
+      <c r="C46" s="8">
         <v>0.74</v>
       </c>
       <c r="D46" s="1">
@@ -1094,7 +2724,7 @@
       <c r="B47" t="s">
         <v>11</v>
       </c>
-      <c r="C47" s="2">
+      <c r="C47" s="8">
         <v>1</v>
       </c>
       <c r="D47" s="1">
@@ -1108,7 +2738,7 @@
       <c r="B48" t="s">
         <v>11</v>
       </c>
-      <c r="C48" s="2">
+      <c r="C48" s="8">
         <v>0.85</v>
       </c>
       <c r="D48" s="1">
@@ -1122,7 +2752,7 @@
       <c r="B49" t="s">
         <v>11</v>
       </c>
-      <c r="C49" s="2">
+      <c r="C49" s="8">
         <v>0.79</v>
       </c>
       <c r="D49" s="1">
@@ -1136,7 +2766,7 @@
       <c r="B50" t="s">
         <v>8</v>
       </c>
-      <c r="C50" s="2">
+      <c r="C50" s="8">
         <v>2</v>
       </c>
       <c r="D50" s="1">
@@ -1150,7 +2780,7 @@
       <c r="B51" t="s">
         <v>8</v>
       </c>
-      <c r="C51" s="2">
+      <c r="C51" s="8">
         <v>2.2999999999999998</v>
       </c>
       <c r="D51" s="1">
@@ -1164,7 +2794,7 @@
       <c r="B52" t="s">
         <v>8</v>
       </c>
-      <c r="C52" s="2">
+      <c r="C52" s="8">
         <v>2.2000000000000002</v>
       </c>
       <c r="D52" s="1">
@@ -1178,7 +2808,7 @@
       <c r="B53" t="s">
         <v>8</v>
       </c>
-      <c r="C53" s="2">
+      <c r="C53" s="8">
         <v>2.1</v>
       </c>
       <c r="D53" s="1">
@@ -1192,7 +2822,7 @@
       <c r="B54" t="s">
         <v>8</v>
       </c>
-      <c r="C54" s="2">
+      <c r="C54" s="8">
         <v>2.4</v>
       </c>
       <c r="D54" s="1">
@@ -1206,7 +2836,7 @@
       <c r="B55" t="s">
         <v>8</v>
       </c>
-      <c r="C55" s="2">
+      <c r="C55" s="8">
         <v>2.4500000000000002</v>
       </c>
       <c r="D55" s="1">
@@ -1220,7 +2850,7 @@
       <c r="B56" t="s">
         <v>8</v>
       </c>
-      <c r="C56" s="2">
+      <c r="C56" s="8">
         <v>2.4</v>
       </c>
       <c r="D56" s="1">
@@ -1234,7 +2864,7 @@
       <c r="B57" t="s">
         <v>8</v>
       </c>
-      <c r="C57" s="2">
+      <c r="C57" s="8">
         <v>2.5</v>
       </c>
       <c r="D57" s="1">
@@ -1248,7 +2878,7 @@
       <c r="B58" t="s">
         <v>8</v>
       </c>
-      <c r="C58" s="2">
+      <c r="C58" s="8">
         <v>2.7</v>
       </c>
       <c r="D58" s="1">
@@ -1262,7 +2892,7 @@
       <c r="B59" t="s">
         <v>8</v>
       </c>
-      <c r="C59" s="2">
+      <c r="C59" s="8">
         <v>2.9</v>
       </c>
       <c r="D59" s="1">
@@ -1276,7 +2906,7 @@
       <c r="B60" t="s">
         <v>8</v>
       </c>
-      <c r="C60" s="2">
+      <c r="C60" s="8">
         <v>2.7</v>
       </c>
       <c r="D60" s="1">
@@ -1290,15 +2920,1690 @@
       <c r="B61" t="s">
         <v>8</v>
       </c>
-      <c r="C61" s="2">
+      <c r="C61" s="8">
         <v>3</v>
       </c>
       <c r="D61" s="1">
         <v>44652</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>4</v>
+      </c>
+      <c r="B62" t="s">
+        <v>12</v>
+      </c>
+      <c r="C62" s="8">
+        <v>14</v>
+      </c>
+      <c r="D62" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>5</v>
+      </c>
+      <c r="B63" t="s">
+        <v>12</v>
+      </c>
+      <c r="C63" s="8">
+        <v>13.5</v>
+      </c>
+      <c r="D63" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>6</v>
+      </c>
+      <c r="B64" t="s">
+        <v>12</v>
+      </c>
+      <c r="C64" s="8">
+        <v>15</v>
+      </c>
+      <c r="D64" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>4</v>
+      </c>
+      <c r="B65" t="s">
+        <v>12</v>
+      </c>
+      <c r="C65" s="8">
+        <v>14.5</v>
+      </c>
+      <c r="D65" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>5</v>
+      </c>
+      <c r="B66" t="s">
+        <v>12</v>
+      </c>
+      <c r="C66" s="8">
+        <v>14</v>
+      </c>
+      <c r="D66" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>6</v>
+      </c>
+      <c r="B67" t="s">
+        <v>12</v>
+      </c>
+      <c r="C67" s="8">
+        <v>15.25</v>
+      </c>
+      <c r="D67" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>4</v>
+      </c>
+      <c r="B68" t="s">
+        <v>13</v>
+      </c>
+      <c r="C68" s="8">
+        <v>10</v>
+      </c>
+      <c r="D68" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>5</v>
+      </c>
+      <c r="B69" t="s">
+        <v>13</v>
+      </c>
+      <c r="C69" s="8">
+        <v>13</v>
+      </c>
+      <c r="D69" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>6</v>
+      </c>
+      <c r="B70" t="s">
+        <v>13</v>
+      </c>
+      <c r="C70" s="8">
+        <v>12.5</v>
+      </c>
+      <c r="D70" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>4</v>
+      </c>
+      <c r="B71" t="s">
+        <v>13</v>
+      </c>
+      <c r="C71" s="8">
+        <v>11</v>
+      </c>
+      <c r="D71" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>5</v>
+      </c>
+      <c r="B72" t="s">
+        <v>13</v>
+      </c>
+      <c r="C72" s="8">
+        <v>13</v>
+      </c>
+      <c r="D72" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>6</v>
+      </c>
+      <c r="B73" t="s">
+        <v>13</v>
+      </c>
+      <c r="C73" s="8">
+        <v>12.75</v>
+      </c>
+      <c r="D73" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>4</v>
+      </c>
+      <c r="B74" t="s">
+        <v>14</v>
+      </c>
+      <c r="C74" s="8">
+        <v>5</v>
+      </c>
+      <c r="D74" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>5</v>
+      </c>
+      <c r="B75" t="s">
+        <v>14</v>
+      </c>
+      <c r="C75" s="8">
+        <v>5</v>
+      </c>
+      <c r="D75" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>6</v>
+      </c>
+      <c r="B76" t="s">
+        <v>14</v>
+      </c>
+      <c r="C76" s="8">
+        <v>6</v>
+      </c>
+      <c r="D76" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>4</v>
+      </c>
+      <c r="B77" t="s">
+        <v>14</v>
+      </c>
+      <c r="C77" s="8">
+        <v>5.5</v>
+      </c>
+      <c r="D77" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>5</v>
+      </c>
+      <c r="B78" t="s">
+        <v>14</v>
+      </c>
+      <c r="C78" s="8">
+        <v>5.25</v>
+      </c>
+      <c r="D78" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>6</v>
+      </c>
+      <c r="B79" t="s">
+        <v>14</v>
+      </c>
+      <c r="C79" s="8">
+        <v>6.25</v>
+      </c>
+      <c r="D79" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>4</v>
+      </c>
+      <c r="B80" t="s">
+        <v>15</v>
+      </c>
+      <c r="C80" s="8">
+        <v>39</v>
+      </c>
+      <c r="D80" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>5</v>
+      </c>
+      <c r="B81" t="s">
+        <v>15</v>
+      </c>
+      <c r="C81" s="8">
+        <v>29</v>
+      </c>
+      <c r="D81" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>6</v>
+      </c>
+      <c r="B82" t="s">
+        <v>15</v>
+      </c>
+      <c r="C82" s="8">
+        <v>38</v>
+      </c>
+      <c r="D82" s="1">
+        <v>44562</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>4</v>
+      </c>
+      <c r="B83" t="s">
+        <v>15</v>
+      </c>
+      <c r="C83" s="8">
+        <v>39</v>
+      </c>
+      <c r="D83" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>5</v>
+      </c>
+      <c r="B84" t="s">
+        <v>15</v>
+      </c>
+      <c r="C84" s="8">
+        <v>31</v>
+      </c>
+      <c r="D84" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>6</v>
+      </c>
+      <c r="B85" t="s">
+        <v>15</v>
+      </c>
+      <c r="C85" s="8">
+        <v>39</v>
+      </c>
+      <c r="D85" s="1">
+        <v>44564</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D59A4F53-9FD0-4853-B2DF-42DEF94E7C50}">
+  <dimension ref="A3:F35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="10.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="8">
+        <v>175.14</v>
+      </c>
+      <c r="C5" s="8">
+        <v>54.72</v>
+      </c>
+      <c r="D5" s="8">
+        <v>56.129999999999995</v>
+      </c>
+      <c r="E5" s="8">
+        <v>57.68</v>
+      </c>
+      <c r="F5" s="8">
+        <v>343.66999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="8">
+        <v>4.25</v>
+      </c>
+      <c r="C6" s="8">
+        <v>4.49</v>
+      </c>
+      <c r="D6" s="8">
+        <v>4.8</v>
+      </c>
+      <c r="E6" s="8">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="F6" s="8">
+        <v>18.43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="C7" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="D7" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="E7" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="F7" s="8">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="8">
+        <v>20.99</v>
+      </c>
+      <c r="C8" s="8">
+        <v>22.99</v>
+      </c>
+      <c r="D8" s="8">
+        <v>22.99</v>
+      </c>
+      <c r="E8" s="8">
+        <v>23.99</v>
+      </c>
+      <c r="F8" s="8">
+        <v>90.96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="8">
+        <v>10.25</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8">
+        <v>10.25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="8">
+        <v>26</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="8">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="C11" s="8">
+        <v>2.4</v>
+      </c>
+      <c r="D11" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="E11" s="8">
+        <v>2.7</v>
+      </c>
+      <c r="F11" s="8">
+        <v>9.8999999999999986</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="8">
+        <v>23</v>
+      </c>
+      <c r="C12" s="8">
+        <v>23.99</v>
+      </c>
+      <c r="D12" s="8">
+        <v>24.99</v>
+      </c>
+      <c r="E12" s="8">
+        <v>25.25</v>
+      </c>
+      <c r="F12" s="8">
+        <v>97.22999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="8">
+        <v>27.5</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="8">
+        <v>60</v>
+      </c>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="8">
+        <v>199.57</v>
+      </c>
+      <c r="C15" s="8">
+        <v>56.53</v>
+      </c>
+      <c r="D15" s="8">
+        <v>58.39</v>
+      </c>
+      <c r="E15" s="8">
+        <v>59.68</v>
+      </c>
+      <c r="F15" s="8">
+        <v>374.16999999999996</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="8">
+        <v>4.99</v>
+      </c>
+      <c r="C16" s="8">
+        <v>5.15</v>
+      </c>
+      <c r="D16" s="8">
+        <v>5.25</v>
+      </c>
+      <c r="E16" s="8">
+        <v>5.35</v>
+      </c>
+      <c r="F16" s="8">
+        <v>20.740000000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="8">
+        <v>0.65</v>
+      </c>
+      <c r="C17" s="8">
+        <v>0.69</v>
+      </c>
+      <c r="D17" s="8">
+        <v>0.74</v>
+      </c>
+      <c r="E17" s="8">
+        <v>0.79</v>
+      </c>
+      <c r="F17" s="8">
+        <v>2.87</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="8">
+        <v>23.99</v>
+      </c>
+      <c r="C18" s="8">
+        <v>24.99</v>
+      </c>
+      <c r="D18" s="8">
+        <v>25.45</v>
+      </c>
+      <c r="E18" s="8">
+        <v>25.79</v>
+      </c>
+      <c r="F18" s="8">
+        <v>100.22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="8">
+        <v>12.25</v>
+      </c>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8">
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="8">
+        <v>25.25</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8">
+        <v>25.25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C21" s="8">
+        <v>2.4500000000000002</v>
+      </c>
+      <c r="D21" s="8">
+        <v>2.7</v>
+      </c>
+      <c r="E21" s="8">
+        <v>3</v>
+      </c>
+      <c r="F21" s="8">
+        <v>10.350000000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="8">
+        <v>22.99</v>
+      </c>
+      <c r="C22" s="8">
+        <v>23.25</v>
+      </c>
+      <c r="D22" s="8">
+        <v>24.25</v>
+      </c>
+      <c r="E22" s="8">
+        <v>24.75</v>
+      </c>
+      <c r="F22" s="8">
+        <v>95.24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="8">
+        <v>30.25</v>
+      </c>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8">
+        <v>30.25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="8">
+        <v>77</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" s="8">
+        <v>193.64</v>
+      </c>
+      <c r="C25" s="8">
+        <v>57.839999999999996</v>
+      </c>
+      <c r="D25" s="8">
+        <v>59.94</v>
+      </c>
+      <c r="E25" s="8">
+        <v>61.129999999999995</v>
+      </c>
+      <c r="F25" s="8">
+        <v>372.54999999999995</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="8">
+        <v>5</v>
+      </c>
+      <c r="C26" s="8">
+        <v>5.25</v>
+      </c>
+      <c r="D26" s="8">
+        <v>5.45</v>
+      </c>
+      <c r="E26" s="8">
+        <v>5.75</v>
+      </c>
+      <c r="F26" s="8">
+        <v>21.45</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="8">
+        <v>0.65</v>
+      </c>
+      <c r="C27" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="D27" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="E27" s="8">
+        <v>1</v>
+      </c>
+      <c r="F27" s="8">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" s="8">
+        <v>22.99</v>
+      </c>
+      <c r="C28" s="8">
+        <v>23.99</v>
+      </c>
+      <c r="D28" s="8">
+        <v>24.25</v>
+      </c>
+      <c r="E28" s="8">
+        <v>24.49</v>
+      </c>
+      <c r="F28" s="8">
+        <v>95.719999999999985</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" s="8">
+        <v>10.5</v>
+      </c>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" s="8">
+        <v>21</v>
+      </c>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31" s="8">
+        <v>2</v>
+      </c>
+      <c r="C31" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="D31" s="8">
+        <v>2.4</v>
+      </c>
+      <c r="E31" s="8">
+        <v>2.9</v>
+      </c>
+      <c r="F31" s="8">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" s="8">
+        <v>25</v>
+      </c>
+      <c r="C32" s="8">
+        <v>25.75</v>
+      </c>
+      <c r="D32" s="8">
+        <v>26.99</v>
+      </c>
+      <c r="E32" s="8">
+        <v>26.99</v>
+      </c>
+      <c r="F32" s="8">
+        <v>104.72999999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B33" s="8">
+        <v>28.5</v>
+      </c>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" s="8">
+        <v>78</v>
+      </c>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" s="8">
+        <v>568.34999999999991</v>
+      </c>
+      <c r="C35" s="8">
+        <v>169.09</v>
+      </c>
+      <c r="D35" s="8">
+        <v>174.46</v>
+      </c>
+      <c r="E35" s="8">
+        <v>178.49</v>
+      </c>
+      <c r="F35" s="8">
+        <v>1090.3900000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7001F8C5-7249-4E0C-B8EA-EBF2F6A75CEA}">
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="11">
+        <v>44562</v>
+      </c>
+      <c r="D4" s="11">
+        <v>44593</v>
+      </c>
+      <c r="E4" s="11">
+        <v>44621</v>
+      </c>
+      <c r="F4" s="11">
+        <v>44652</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="8">
+        <v>4.25</v>
+      </c>
+      <c r="D5" s="8">
+        <v>4.49</v>
+      </c>
+      <c r="E5" s="8">
+        <v>4.8</v>
+      </c>
+      <c r="F5" s="8">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="G5" s="13">
+        <f>SUM(C5:F5)</f>
+        <v>18.43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="D6" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="E6" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="F6" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="G6" s="13">
+        <f t="shared" ref="G6:G13" si="0">SUM(C6:F6)</f>
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="8">
+        <v>20.99</v>
+      </c>
+      <c r="D7" s="8">
+        <v>22.99</v>
+      </c>
+      <c r="E7" s="8">
+        <v>22.99</v>
+      </c>
+      <c r="F7" s="8">
+        <v>23.99</v>
+      </c>
+      <c r="G7" s="13">
+        <f t="shared" si="0"/>
+        <v>90.96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="8">
+        <v>10.25</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="13">
+        <f t="shared" si="0"/>
+        <v>10.25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="8">
+        <v>26</v>
+      </c>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="13">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="8">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D10" s="8">
+        <v>2.4</v>
+      </c>
+      <c r="E10" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="F10" s="8">
+        <v>2.7</v>
+      </c>
+      <c r="G10" s="13">
+        <f t="shared" si="0"/>
+        <v>9.8999999999999986</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="8">
+        <v>23</v>
+      </c>
+      <c r="D11" s="8">
+        <v>23.99</v>
+      </c>
+      <c r="E11" s="8">
+        <v>24.99</v>
+      </c>
+      <c r="F11" s="8">
+        <v>25.25</v>
+      </c>
+      <c r="G11" s="13">
+        <f t="shared" si="0"/>
+        <v>97.22999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="8">
+        <v>27.5</v>
+      </c>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="13">
+        <f t="shared" si="0"/>
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="8">
+        <v>60</v>
+      </c>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="13">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B14" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="15">
+        <f>SUM(C5:C13)</f>
+        <v>175.14</v>
+      </c>
+      <c r="D14" s="15">
+        <f t="shared" ref="D14:G14" si="1">SUM(D5:D13)</f>
+        <v>54.72</v>
+      </c>
+      <c r="E14" s="15">
+        <f t="shared" si="1"/>
+        <v>56.129999999999995</v>
+      </c>
+      <c r="F14" s="15">
+        <f t="shared" si="1"/>
+        <v>57.68</v>
+      </c>
+      <c r="G14" s="16">
+        <f t="shared" si="1"/>
+        <v>343.66999999999996</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="8">
+        <v>4.99</v>
+      </c>
+      <c r="D15" s="8">
+        <v>5.15</v>
+      </c>
+      <c r="E15" s="8">
+        <v>5.25</v>
+      </c>
+      <c r="F15" s="8">
+        <v>5.35</v>
+      </c>
+      <c r="G15" s="13">
+        <f>SUM(C15:F15)</f>
+        <v>20.740000000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="8">
+        <v>0.65</v>
+      </c>
+      <c r="D16" s="8">
+        <v>0.69</v>
+      </c>
+      <c r="E16" s="8">
+        <v>0.74</v>
+      </c>
+      <c r="F16" s="8">
+        <v>0.79</v>
+      </c>
+      <c r="G16" s="13">
+        <f t="shared" ref="G16:G23" si="2">SUM(C16:F16)</f>
+        <v>2.87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="8">
+        <v>23.99</v>
+      </c>
+      <c r="D17" s="8">
+        <v>24.99</v>
+      </c>
+      <c r="E17" s="8">
+        <v>25.45</v>
+      </c>
+      <c r="F17" s="8">
+        <v>25.79</v>
+      </c>
+      <c r="G17" s="13">
+        <f t="shared" si="2"/>
+        <v>100.22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="8">
+        <v>12.25</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="13">
+        <f t="shared" si="2"/>
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="8">
+        <v>25.25</v>
+      </c>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="13">
+        <f t="shared" si="2"/>
+        <v>25.25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D20" s="8">
+        <v>2.4500000000000002</v>
+      </c>
+      <c r="E20" s="8">
+        <v>2.7</v>
+      </c>
+      <c r="F20" s="8">
+        <v>3</v>
+      </c>
+      <c r="G20" s="13">
+        <f t="shared" si="2"/>
+        <v>10.350000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="8">
+        <v>22.99</v>
+      </c>
+      <c r="D21" s="8">
+        <v>23.25</v>
+      </c>
+      <c r="E21" s="8">
+        <v>24.25</v>
+      </c>
+      <c r="F21" s="8">
+        <v>24.75</v>
+      </c>
+      <c r="G21" s="13">
+        <f t="shared" si="2"/>
+        <v>95.24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="8">
+        <v>30.25</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="13">
+        <f t="shared" si="2"/>
+        <v>30.25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="8">
+        <v>77</v>
+      </c>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="13">
+        <f t="shared" si="2"/>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B24" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="15">
+        <f>SUM(C15:C23)</f>
+        <v>199.57</v>
+      </c>
+      <c r="D24" s="15">
+        <f t="shared" ref="D24:G24" si="3">SUM(D15:D23)</f>
+        <v>56.53</v>
+      </c>
+      <c r="E24" s="15">
+        <f t="shared" si="3"/>
+        <v>58.39</v>
+      </c>
+      <c r="F24" s="15">
+        <f t="shared" si="3"/>
+        <v>59.68</v>
+      </c>
+      <c r="G24" s="16">
+        <f t="shared" si="3"/>
+        <v>374.16999999999996</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" s="8">
+        <v>5</v>
+      </c>
+      <c r="D25" s="8">
+        <v>5.25</v>
+      </c>
+      <c r="E25" s="8">
+        <v>5.45</v>
+      </c>
+      <c r="F25" s="8">
+        <v>5.75</v>
+      </c>
+      <c r="G25" s="13">
+        <f>SUM(C25:F25)</f>
+        <v>21.45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" s="8">
+        <v>0.65</v>
+      </c>
+      <c r="D26" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="E26" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="F26" s="8">
+        <v>1</v>
+      </c>
+      <c r="G26" s="13">
+        <f t="shared" ref="G26:G33" si="4">SUM(C26:F26)</f>
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="8">
+        <v>22.99</v>
+      </c>
+      <c r="D27" s="8">
+        <v>23.99</v>
+      </c>
+      <c r="E27" s="8">
+        <v>24.25</v>
+      </c>
+      <c r="F27" s="8">
+        <v>24.49</v>
+      </c>
+      <c r="G27" s="13">
+        <f t="shared" si="4"/>
+        <v>95.719999999999985</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="8">
+        <v>10.5</v>
+      </c>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="13">
+        <f t="shared" si="4"/>
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="8">
+        <v>21</v>
+      </c>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="13">
+        <f t="shared" si="4"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="8">
+        <v>2</v>
+      </c>
+      <c r="D30" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="E30" s="8">
+        <v>2.4</v>
+      </c>
+      <c r="F30" s="8">
+        <v>2.9</v>
+      </c>
+      <c r="G30" s="13">
+        <f t="shared" si="4"/>
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" s="8">
+        <v>25</v>
+      </c>
+      <c r="D31" s="8">
+        <v>25.75</v>
+      </c>
+      <c r="E31" s="8">
+        <v>26.99</v>
+      </c>
+      <c r="F31" s="8">
+        <v>26.99</v>
+      </c>
+      <c r="G31" s="13">
+        <f t="shared" si="4"/>
+        <v>104.72999999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" s="8">
+        <v>28.5</v>
+      </c>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="13">
+        <f t="shared" si="4"/>
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" s="8">
+        <v>78</v>
+      </c>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="13">
+        <f t="shared" si="4"/>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B34" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" s="15">
+        <f>SUM(C25:C33)</f>
+        <v>193.64</v>
+      </c>
+      <c r="D34" s="15">
+        <f t="shared" ref="D34:G34" si="5">SUM(D25:D33)</f>
+        <v>57.839999999999996</v>
+      </c>
+      <c r="E34" s="15">
+        <f t="shared" si="5"/>
+        <v>59.94</v>
+      </c>
+      <c r="F34" s="15">
+        <f t="shared" si="5"/>
+        <v>61.129999999999995</v>
+      </c>
+      <c r="G34" s="16">
+        <f t="shared" si="5"/>
+        <v>372.54999999999995</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B35" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C35" s="18">
+        <f>SUM(C14,C24,C34)</f>
+        <v>568.34999999999991</v>
+      </c>
+      <c r="D35" s="18">
+        <f t="shared" ref="D35:G35" si="6">SUM(D14,D24,D34)</f>
+        <v>169.09</v>
+      </c>
+      <c r="E35" s="18">
+        <f t="shared" si="6"/>
+        <v>174.45999999999998</v>
+      </c>
+      <c r="F35" s="18">
+        <f t="shared" si="6"/>
+        <v>178.49</v>
+      </c>
+      <c r="G35" s="18">
+        <f t="shared" si="6"/>
+        <v>1090.3899999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>